<commit_message>
fix: rename query IDs to standard format Q3_001–Q3_018 and Q4_001–Q4_014
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/data/evaluation/potential_queries/queries_type_3.xlsx
+++ b/data/evaluation/potential_queries/queries_type_3.xlsx
@@ -469,11 +469,13 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Deep_Query_1</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>3</v>
+          <t>Q3_001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -495,11 +497,13 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Deep_Query_2</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>3</v>
+          <t>Q3_002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -521,11 +525,13 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Deep_Query_3</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>3</v>
+          <t>Q3_003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -547,11 +553,13 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Deep_Query_4</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>3</v>
+          <t>Q3_004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -573,11 +581,13 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Deep_Query_5</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>3</v>
+          <t>Q3_005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -599,11 +609,13 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Deep_Query_11</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>3</v>
+          <t>Q3_006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -625,11 +637,13 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Deep_Query_12</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>3</v>
+          <t>Q3_007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -651,11 +665,13 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Deep_Query_13</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>3</v>
+          <t>Q3_008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -677,11 +693,13 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Deep_Query_14</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>3</v>
+          <t>Q3_009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -703,11 +721,13 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Deep_Query_15</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>3</v>
+          <t>Q3_010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -729,11 +749,13 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Deep_Query_21</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>3</v>
+          <t>Q3_011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -755,11 +777,13 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Deep_Query_24</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>3</v>
+          <t>Q3_012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -781,11 +805,13 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Deep_Query_25</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>3</v>
+          <t>Q3_013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -807,11 +833,13 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Deep_Query_28</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>3</v>
+          <t>Q3_014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -833,11 +861,13 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Deep_Query_29</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>3</v>
+          <t>Q3_015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -859,11 +889,13 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Deep_Query_30</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>3</v>
+          <t>Q3_016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -885,11 +917,13 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Deep_Query_31</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>3</v>
+          <t>Q3_017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -911,11 +945,13 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Deep_Query_32</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>3</v>
+          <t>Q3_018</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>

</xml_diff>